<commit_message>
EGCH 01-09-2026 edition: print the weighted central, read the bibliography from the register
- The valuation summary, READ FIRST, section 1.5 and the Summary sheet now
  carry the weighted central (EGP 3.76) with its weights stated, inside the
  published field, never as a point target.
- The bibliography's market table reads the register exclusively; the stale
  live_data.json read and the unconsumed erp_cds input are gone, so the
  superseded 9.42% CDS premium no longer prints anywhere.
- prose_check.py matches prose figures against consumed register values only.
- Section 1.8 states the FX-leg disclosure in the study's own words with the
  floored alternative priced beside it; section 3 adds record strength and
  width ratio from the band record; terminal cost-of-debt labels computed.

Fair value unchanged: 0.00 / 3.76 / 15.47.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUBWMwER6i6M5VJH7eDW4Q
</commit_message>
<xml_diff>
--- a/engine/egch_study/EGCH_Valuation_Model_01092026.xlsx
+++ b/engine/egch_study/EGCH_Valuation_Model_01092026.xlsx
@@ -3437,7 +3437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3766,6 +3766,82 @@
       <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Terminal value as a share of enterprise value is reported beside the cash-flow lens on the DCF sheet, in both columns, because on this company it is the number that decides the answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>THE WEIGHTED CENTRAL INSIDE THE FIELD — stated weights, reading the lens cells above</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Weight: cash flow, programme carried through</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Weight: relative multiples</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Weight: normalised earnings power</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Weight: book value and sustainable return</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Weighted central (EGP/share)</t>
+        </is>
+      </c>
+      <c r="B38" s="11">
+        <f>B34*B5+B35*B7+B36*B8+B37*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Against spot</t>
+        </is>
+      </c>
+      <c r="B39" s="8">
+        <f>B38/$B$14-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Only the carried-through side of the cash-flow lens enters the weighting (the company's stated plan); the stopped reading is the contested judgement above, published beside it and never averaged in. Bear and full are the field's floor and ceiling, never the weighted extremes.</t>
         </is>
       </c>
     </row>

</xml_diff>